<commit_message>
dynamic w static rows missing: certificate
Co-authored-by: hikusama <leomessi25k@gmail.com>
</commit_message>
<xml_diff>
--- a/src/UI-Admin/contents/sf10/sf10.xlsx
+++ b/src/UI-Admin/contents/sf10/sf10.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\sta.MariaSystem\src\UI-Admin\contents\sf10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23402E98-13A1-4A60-B99A-0924CCC56ACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{906CB6E4-5D85-42EE-85E1-F336ED180B8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{2526813D-373B-47EA-9554-6CA2D7102D83}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{2526813D-373B-47EA-9554-6CA2D7102D83}"/>
   </bookViews>
   <sheets>
     <sheet name="Front" sheetId="1" r:id="rId1"/>

</xml_diff>